<commit_message>
docs(int): format the full-setup workbook (headers, borders, bands, links back)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/samples/full-setup/Slotwise-Full-Setup.xlsx
+++ b/docs/samples/full-setup/Slotwise-Full-Setup.xlsx
@@ -691,7 +691,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="212">
   <si>
     <t>Slotwise full setup: Civil Engineering for the Demo Institute (fictional data)</t>
   </si>
@@ -795,6 +795,12 @@
     <t>Teachers for every lecture, tutorial and lab of CE S1. Labs are taught per lab group. Choose the current term when you upload.</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
+    <t>Key: dark headers are the import columns; a yellow underline marks a required column; hover a header for what to type.</t>
+  </si>
+  <si>
     <t>Code</t>
   </si>
   <si>
@@ -802,6 +808,9 @@
   </si>
   <si>
     <t>Kind</t>
+  </si>
+  <si>
+    <t>← Start here</t>
   </si>
   <si>
     <t>CE</t>
@@ -1324,7 +1333,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -1334,7 +1343,8 @@
     </font>
     <font>
       <b/>
-      <sz val="14"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="16"/>
     </font>
     <font>
       <b/>
@@ -1343,8 +1353,16 @@
       <u/>
       <color rgb="FF1D4ED8"/>
     </font>
+    <font>
+      <i/>
+      <color rgb="FF555555"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1353,11 +1371,16 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
+        <fgColor rgb="FF1E3A8A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEEF2FF"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -1365,19 +1388,69 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD1D5DB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD1D5DB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFF5B700"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF1E3A8A"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1717,7 +1790,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E12"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -1727,198 +1803,213 @@
     <col min="5" max="5" width="80" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" ht="30" customHeight="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-    </row>
-    <row r="2" ht="34" customHeight="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+    </row>
+    <row r="2" ht="36" customHeight="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-    </row>
-    <row r="3" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="4" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4">
+      <c r="A4" s="5">
         <v>1</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="5">
         <v>1</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5">
+      <c r="A5" s="5">
         <v>2</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="5">
         <v>1</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="5" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6">
+      <c r="A6" s="5">
         <v>3</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="5">
         <v>4</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="5" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7">
+      <c r="A7" s="5">
         <v>4</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="5">
         <v>4</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="5" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8">
+      <c r="A8" s="5">
         <v>5</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="5">
         <v>5</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="5" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9">
+      <c r="A9" s="5">
         <v>6</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="5">
         <v>1</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="5" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10">
+      <c r="A10" s="5">
         <v>7</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="5">
         <v>10</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="5" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11">
+      <c r="A11" s="5">
         <v>8</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="5">
         <v>2</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="5" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12">
+      <c r="A12" s="5">
         <v>9</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="5">
         <v>8</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="5" t="s">
         <v>33</v>
       </c>
     </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A14:E14"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B4" r:id="rId1" location="#'Departments'!A1"/>
@@ -1931,14 +2022,16 @@
     <hyperlink ref="B11" r:id="rId8" location="#'Holidays'!A1"/>
     <hyperlink ref="B12" r:id="rId9" location="#'Who teaches what'!A1"/>
   </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G200"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:I200"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -1948,175 +2041,182 @@
     <col min="7" max="7" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
-        <v>204</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>205</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>206</v>
-      </c>
-      <c r="G1" s="3" t="s">
+    <row r="1" ht="22" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
         <v>207</v>
       </c>
+      <c r="B1" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="I1" s="10" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>208</v>
-      </c>
-      <c r="B2" t="s">
-        <v>148</v>
-      </c>
-      <c r="D2" t="s">
-        <v>70</v>
-      </c>
-      <c r="E2" t="s">
-        <v>58</v>
-      </c>
-      <c r="F2" t="s">
-        <v>115</v>
+      <c r="A2" s="11" t="s">
+        <v>211</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>208</v>
-      </c>
-      <c r="B3" t="s">
-        <v>148</v>
-      </c>
-      <c r="D3" t="s">
-        <v>70</v>
-      </c>
-      <c r="E3" t="s">
-        <v>59</v>
-      </c>
-      <c r="F3" t="s">
-        <v>115</v>
+      <c r="A3" s="12" t="s">
+        <v>211</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>208</v>
-      </c>
-      <c r="B4" t="s">
-        <v>148</v>
-      </c>
-      <c r="D4" t="s">
-        <v>74</v>
-      </c>
-      <c r="E4" t="s">
-        <v>58</v>
-      </c>
-      <c r="F4" t="s">
-        <v>121</v>
+      <c r="A4" s="11" t="s">
+        <v>211</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>208</v>
-      </c>
-      <c r="B5" t="s">
-        <v>148</v>
-      </c>
-      <c r="C5" t="s">
-        <v>158</v>
-      </c>
-      <c r="D5" t="s">
-        <v>74</v>
-      </c>
-      <c r="E5" t="s">
-        <v>60</v>
-      </c>
-      <c r="F5" t="s">
-        <v>121</v>
+      <c r="A5" s="12" t="s">
+        <v>211</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>161</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>208</v>
-      </c>
-      <c r="B6" t="s">
-        <v>148</v>
-      </c>
-      <c r="C6" t="s">
-        <v>179</v>
-      </c>
-      <c r="D6" t="s">
-        <v>74</v>
-      </c>
-      <c r="E6" t="s">
-        <v>60</v>
-      </c>
-      <c r="F6" t="s">
-        <v>126</v>
+      <c r="A6" s="11" t="s">
+        <v>211</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>182</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>208</v>
-      </c>
-      <c r="B7" t="s">
-        <v>148</v>
-      </c>
-      <c r="D7" t="s">
-        <v>78</v>
-      </c>
-      <c r="E7" t="s">
-        <v>58</v>
-      </c>
-      <c r="F7" t="s">
-        <v>131</v>
+      <c r="A7" s="12" t="s">
+        <v>211</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="C7" s="12"/>
+      <c r="D7" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>208</v>
-      </c>
-      <c r="B8" t="s">
-        <v>148</v>
-      </c>
-      <c r="C8" t="s">
-        <v>158</v>
-      </c>
-      <c r="D8" t="s">
-        <v>81</v>
-      </c>
-      <c r="E8" t="s">
-        <v>60</v>
-      </c>
-      <c r="F8" t="s">
-        <v>136</v>
+      <c r="A8" s="11" t="s">
+        <v>211</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>208</v>
-      </c>
-      <c r="B9" t="s">
-        <v>148</v>
-      </c>
-      <c r="C9" t="s">
-        <v>179</v>
-      </c>
-      <c r="D9" t="s">
-        <v>81</v>
-      </c>
-      <c r="E9" t="s">
-        <v>60</v>
-      </c>
-      <c r="F9" t="s">
-        <v>126</v>
+      <c r="A9" s="12" t="s">
+        <v>211</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>182</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="F9" s="12" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="10" spans="4:6" x14ac:dyDescent="0.25"/>
@@ -2331,15 +2431,20 @@
       <formula1>'Faculty'!$C$2:$C$500</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-  <legacyDrawing r:id="rId2"/>
+  <hyperlinks>
+    <hyperlink ref="I1" r:id="rId1" location="#'Start here'!A1"/>
+  </hyperlinks>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C200"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:E200"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -2347,26 +2452,29 @@
     <col min="3" max="3" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="C1" s="3" t="s">
+    <row r="1" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
         <v>36</v>
       </c>
+      <c r="B1" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C2" t="s">
-        <v>39</v>
+      <c r="A2" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="3:3" x14ac:dyDescent="0.25"/>
@@ -2576,15 +2684,20 @@
       <formula1>"Teaching,Service"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-  <legacyDrawing r:id="rId2"/>
+  <hyperlinks>
+    <hyperlink ref="E1" r:id="rId1" location="#'Start here'!A1"/>
+  </hyperlinks>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I200"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:K200"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="18" customWidth="1"/>
@@ -2597,59 +2710,63 @@
     <col min="9" max="9" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+    <row r="1" ht="22" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="K1" s="10" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="D2" s="11">
+        <v>8</v>
+      </c>
+      <c r="E2" s="11">
+        <v>3</v>
+      </c>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="H2" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="C1" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D2">
-        <v>8</v>
-      </c>
-      <c r="E2">
-        <v>3</v>
-      </c>
-      <c r="G2" t="s">
-        <v>37</v>
-      </c>
-      <c r="H2" t="s">
-        <v>38</v>
-      </c>
-      <c r="I2" t="s">
-        <v>37</v>
+      <c r="I2" s="11" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="3:9" x14ac:dyDescent="0.25"/>
@@ -2865,15 +2982,20 @@
       <formula1>'Departments'!$A$2:$A$500</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-  <legacyDrawing r:id="rId2"/>
+  <hyperlinks>
+    <hyperlink ref="K1" r:id="rId1" location="#'Start here'!A1"/>
+  </hyperlinks>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q200"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:S200"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="13" customWidth="1"/>
@@ -2891,233 +3013,248 @@
     <col min="17" max="17" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+    <row r="1" ht="22" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="K1" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="L1" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="M1" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="N1" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="O1" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="P1" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q1" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="S1" s="10" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A2" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="B1" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="M1" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="O1" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="P1" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="Q1" s="3" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C2">
+      <c r="B2" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C2" s="11">
         <v>1</v>
       </c>
-      <c r="D2" t="s">
-        <v>70</v>
-      </c>
-      <c r="E2" t="s">
-        <v>71</v>
-      </c>
-      <c r="F2" t="s">
+      <c r="D2" s="11" t="s">
+        <v>73</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="G2" s="11">
+        <v>3</v>
+      </c>
+      <c r="H2" s="11">
+        <v>1</v>
+      </c>
+      <c r="I2" s="11">
+        <v>0</v>
+      </c>
+      <c r="J2" s="11"/>
+      <c r="K2" s="11">
+        <v>45</v>
+      </c>
+      <c r="L2" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="M2" s="11"/>
+      <c r="N2" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="O2" s="11"/>
+      <c r="P2" s="11"/>
+      <c r="Q2" s="11" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="B3" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="G2">
+      <c r="C3" s="12">
+        <v>1</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="G3" s="12">
         <v>3</v>
       </c>
-      <c r="H2">
+      <c r="H3" s="12">
+        <v>0</v>
+      </c>
+      <c r="I3" s="12">
+        <v>2</v>
+      </c>
+      <c r="J3" s="12"/>
+      <c r="K3" s="12">
+        <v>45</v>
+      </c>
+      <c r="L3" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="M3" s="12"/>
+      <c r="N3" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="O3" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="P3" s="12">
+        <v>2</v>
+      </c>
+      <c r="Q3" s="12" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A4" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C4" s="11">
         <v>1</v>
       </c>
-      <c r="I2">
+      <c r="D4" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="G4" s="11">
+        <v>3</v>
+      </c>
+      <c r="H4" s="11">
         <v>0</v>
       </c>
-      <c r="K2">
-        <v>45</v>
-      </c>
-      <c r="L2" t="s">
-        <v>73</v>
-      </c>
-      <c r="N2" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>49</v>
-      </c>
-      <c r="B3" t="s">
-        <v>69</v>
-      </c>
-      <c r="C3">
+      <c r="I4" s="11">
+        <v>0</v>
+      </c>
+      <c r="J4" s="11"/>
+      <c r="K4" s="11">
+        <v>42</v>
+      </c>
+      <c r="L4" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="M4" s="11"/>
+      <c r="N4" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="O4" s="11"/>
+      <c r="P4" s="11"/>
+      <c r="Q4" s="11" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5" s="12">
         <v>1</v>
       </c>
-      <c r="D3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E3" t="s">
-        <v>75</v>
-      </c>
-      <c r="F3" t="s">
-        <v>76</v>
-      </c>
-      <c r="G3">
-        <v>3</v>
-      </c>
-      <c r="H3">
+      <c r="D5" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="G5" s="12">
         <v>0</v>
       </c>
-      <c r="I3">
+      <c r="H5" s="12">
+        <v>0</v>
+      </c>
+      <c r="I5" s="12">
         <v>2</v>
       </c>
-      <c r="K3">
-        <v>45</v>
-      </c>
-      <c r="L3" t="s">
-        <v>73</v>
-      </c>
-      <c r="N3" t="s">
-        <v>37</v>
-      </c>
-      <c r="O3" t="s">
-        <v>77</v>
-      </c>
-      <c r="P3">
+      <c r="J5" s="12"/>
+      <c r="K5" s="12">
+        <v>28</v>
+      </c>
+      <c r="L5" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="M5" s="12"/>
+      <c r="N5" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="O5" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="P5" s="12">
         <v>2</v>
       </c>
-      <c r="Q3" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B4" t="s">
-        <v>69</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="D4" t="s">
-        <v>78</v>
-      </c>
-      <c r="E4" t="s">
-        <v>79</v>
-      </c>
-      <c r="F4" t="s">
-        <v>80</v>
-      </c>
-      <c r="G4">
-        <v>3</v>
-      </c>
-      <c r="H4">
-        <v>0</v>
-      </c>
-      <c r="I4">
-        <v>0</v>
-      </c>
-      <c r="K4">
-        <v>42</v>
-      </c>
-      <c r="L4" t="s">
-        <v>73</v>
-      </c>
-      <c r="N4" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>49</v>
-      </c>
-      <c r="B5" t="s">
-        <v>69</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5" t="s">
-        <v>81</v>
-      </c>
-      <c r="E5" t="s">
-        <v>82</v>
-      </c>
-      <c r="F5" t="s">
-        <v>83</v>
-      </c>
-      <c r="G5">
-        <v>0</v>
-      </c>
-      <c r="H5">
-        <v>0</v>
-      </c>
-      <c r="I5">
-        <v>2</v>
-      </c>
-      <c r="K5">
-        <v>28</v>
-      </c>
-      <c r="L5" t="s">
-        <v>84</v>
-      </c>
-      <c r="N5" t="s">
-        <v>37</v>
-      </c>
-      <c r="O5" t="s">
-        <v>85</v>
-      </c>
-      <c r="P5">
-        <v>2</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>37</v>
+      <c r="Q5" s="12" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="12:14" x14ac:dyDescent="0.25"/>
@@ -3330,15 +3467,20 @@
       <formula1>'Departments'!$A$2:$A$500</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-  <legacyDrawing r:id="rId2"/>
+  <hyperlinks>
+    <hyperlink ref="S1" r:id="rId1" location="#'Start here'!A1"/>
+  </hyperlinks>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L200"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:N200"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -3353,173 +3495,183 @@
     <col min="12" max="12" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="B1" s="5" t="s">
+    <row r="1" ht="22" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="K1" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="L1" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="N1" s="10" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="C2" s="11">
+        <v>0</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11">
+        <v>10</v>
+      </c>
+      <c r="G2" s="11">
+        <v>6</v>
+      </c>
+      <c r="H2" s="11"/>
+      <c r="I2" s="11">
+        <v>1</v>
+      </c>
+      <c r="J2" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="K2" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="L2" s="11" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="C3" s="12">
+        <v>1</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12">
+        <v>10</v>
+      </c>
+      <c r="G3" s="12">
+        <v>6</v>
+      </c>
+      <c r="H3" s="12"/>
+      <c r="I3" s="12">
+        <v>1</v>
+      </c>
+      <c r="J3" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="K3" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="L3" s="12" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="C4" s="11">
+        <v>1</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="E4" s="11"/>
+      <c r="F4" s="11">
+        <v>5</v>
+      </c>
+      <c r="G4" s="11">
+        <v>6</v>
+      </c>
+      <c r="H4" s="11"/>
+      <c r="I4" s="11">
+        <v>1</v>
+      </c>
+      <c r="J4" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="K4" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="L4" s="11" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="C5" s="12">
+        <v>0</v>
+      </c>
+      <c r="D5" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="F1" s="3" t="s">
+      <c r="E5" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="F5" s="12">
+        <v>6</v>
+      </c>
+      <c r="G5" s="12">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>95</v>
-      </c>
-      <c r="B2" t="s">
-        <v>96</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-      <c r="D2" t="s">
-        <v>97</v>
-      </c>
-      <c r="F2">
-        <v>10</v>
-      </c>
-      <c r="G2">
-        <v>6</v>
-      </c>
-      <c r="I2">
+      <c r="H5" s="12"/>
+      <c r="I5" s="12">
         <v>1</v>
       </c>
-      <c r="J2" t="s">
-        <v>37</v>
-      </c>
-      <c r="K2" t="s">
-        <v>98</v>
-      </c>
-      <c r="L2" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>99</v>
-      </c>
-      <c r="B3" t="s">
-        <v>96</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3" t="s">
-        <v>97</v>
-      </c>
-      <c r="F3">
-        <v>10</v>
-      </c>
-      <c r="G3">
-        <v>6</v>
-      </c>
-      <c r="I3">
-        <v>1</v>
-      </c>
-      <c r="J3" t="s">
-        <v>37</v>
-      </c>
-      <c r="K3" t="s">
-        <v>98</v>
-      </c>
-      <c r="L3" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="J5" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="K5" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="L5" s="12" t="s">
         <v>101</v>
-      </c>
-      <c r="B4" t="s">
-        <v>96</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="D4" t="s">
-        <v>102</v>
-      </c>
-      <c r="F4">
-        <v>5</v>
-      </c>
-      <c r="G4">
-        <v>6</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-      <c r="J4" t="s">
-        <v>37</v>
-      </c>
-      <c r="K4" t="s">
-        <v>98</v>
-      </c>
-      <c r="L4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>103</v>
-      </c>
-      <c r="B5" t="s">
-        <v>96</v>
-      </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-      <c r="D5" t="s">
-        <v>84</v>
-      </c>
-      <c r="E5" t="s">
-        <v>104</v>
-      </c>
-      <c r="F5">
-        <v>6</v>
-      </c>
-      <c r="G5">
-        <v>5</v>
-      </c>
-      <c r="I5">
-        <v>1</v>
-      </c>
-      <c r="J5" t="s">
-        <v>37</v>
-      </c>
-      <c r="K5" t="s">
-        <v>100</v>
-      </c>
-      <c r="L5" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="6" spans="4:12" x14ac:dyDescent="0.25"/>
@@ -3738,15 +3890,20 @@
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-  <legacyDrawing r:id="rId2"/>
+  <hyperlinks>
+    <hyperlink ref="N1" r:id="rId1" location="#'Start here'!A1"/>
+  </hyperlinks>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J200"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:L200"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -3760,180 +3917,188 @@
     <col min="10" max="10" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="E1" s="5" t="s">
+    <row r="1" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
         <v>108</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="B1" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C1" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="G1" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="H1" s="3" t="s">
+      <c r="D1" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="E1" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="F1" s="9" t="s">
         <v>112</v>
       </c>
+      <c r="G1" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="L1" s="10" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>113</v>
-      </c>
-      <c r="B2" t="s">
-        <v>114</v>
-      </c>
-      <c r="C2" t="s">
-        <v>115</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="A2" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="E2" t="s">
+      <c r="B2" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="F2" t="s">
+      <c r="C2" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="G2" t="s">
-        <v>37</v>
-      </c>
-      <c r="I2">
+      <c r="D2" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="H2" s="11"/>
+      <c r="I2" s="11">
         <v>4</v>
       </c>
-      <c r="J2">
+      <c r="J2" s="11">
         <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>119</v>
-      </c>
-      <c r="B3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="A3" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="E3" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="F3" s="12" t="s">
         <v>121</v>
       </c>
-      <c r="D3" t="s">
-        <v>122</v>
-      </c>
-      <c r="E3" t="s">
-        <v>123</v>
-      </c>
-      <c r="F3" t="s">
-        <v>118</v>
-      </c>
-      <c r="G3" t="s">
-        <v>37</v>
-      </c>
-      <c r="I3">
+      <c r="G3" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="H3" s="12"/>
+      <c r="I3" s="12">
         <v>5</v>
       </c>
-      <c r="J3">
+      <c r="J3" s="12">
         <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>124</v>
-      </c>
-      <c r="B4" t="s">
-        <v>125</v>
-      </c>
-      <c r="C4" t="s">
-        <v>126</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="A4" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="E4" t="s">
+      <c r="B4" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="F4" t="s">
-        <v>118</v>
-      </c>
-      <c r="G4" t="s">
-        <v>37</v>
-      </c>
-      <c r="I4">
+      <c r="C4" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>131</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>121</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="H4" s="11"/>
+      <c r="I4" s="11">
         <v>5</v>
       </c>
-      <c r="J4">
+      <c r="J4" s="11">
         <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>129</v>
-      </c>
-      <c r="B5" t="s">
-        <v>130</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="A5" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="E5" s="12" t="s">
         <v>131</v>
       </c>
-      <c r="D5" t="s">
-        <v>132</v>
-      </c>
-      <c r="E5" t="s">
-        <v>128</v>
-      </c>
-      <c r="F5" t="s">
-        <v>133</v>
-      </c>
-      <c r="G5" t="s">
-        <v>37</v>
-      </c>
-      <c r="I5">
+      <c r="F5" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="H5" s="12"/>
+      <c r="I5" s="12">
         <v>4</v>
       </c>
-      <c r="J5">
+      <c r="J5" s="12">
         <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>134</v>
-      </c>
-      <c r="B6" t="s">
-        <v>135</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="A6" s="11" t="s">
+        <v>137</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="F6" s="11" t="s">
         <v>136</v>
       </c>
-      <c r="D6" t="s">
-        <v>137</v>
-      </c>
-      <c r="E6" t="s">
-        <v>138</v>
-      </c>
-      <c r="F6" t="s">
-        <v>133</v>
-      </c>
-      <c r="G6" t="s">
-        <v>37</v>
-      </c>
-      <c r="I6">
+      <c r="G6" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11">
         <v>5</v>
       </c>
-      <c r="J6">
+      <c r="J6" s="11">
         <v>18</v>
       </c>
     </row>
@@ -4152,15 +4317,20 @@
       <formula1>'Departments'!$A$2:$A$500</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-  <legacyDrawing r:id="rId2"/>
+  <hyperlinks>
+    <hyperlink ref="L1" r:id="rId1" location="#'Start here'!A1"/>
+  </hyperlinks>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J200"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:L200"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -4174,68 +4344,71 @@
     <col min="10" max="10" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+    <row r="1" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="L1" s="10" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C2">
+      <c r="B2" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" s="11">
         <v>2026</v>
       </c>
-      <c r="D2" t="s">
-        <v>147</v>
-      </c>
-      <c r="E2" t="s">
-        <v>69</v>
-      </c>
-      <c r="F2" t="s">
-        <v>148</v>
-      </c>
-      <c r="G2">
+      <c r="D2" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="G2" s="11">
         <v>60</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="11">
         <v>2</v>
       </c>
-      <c r="I2" t="s">
-        <v>149</v>
-      </c>
-      <c r="J2" t="s">
-        <v>95</v>
+      <c r="I2" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="J2" s="11" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="3" spans="4:10" x14ac:dyDescent="0.25"/>
@@ -4451,15 +4624,20 @@
       <formula1>'Rooms'!$A$2:$A$500</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-  <legacyDrawing r:id="rId2"/>
+  <hyperlinks>
+    <hyperlink ref="L1" r:id="rId1" location="#'Start here'!A1"/>
+  </hyperlinks>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K200"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:M200"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
@@ -4474,359 +4652,372 @@
     <col min="11" max="11" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+    <row r="1" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="K1" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="M1" s="10" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="H2" s="11">
+        <v>2026</v>
+      </c>
+      <c r="I2" s="11" t="s">
         <v>150</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="J2" s="11" t="s">
         <v>151</v>
       </c>
-      <c r="C1" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>152</v>
-      </c>
-      <c r="F1" s="5" t="s">
+      <c r="K2" s="11" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
+        <v>162</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>164</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>165</v>
+      </c>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="G1" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>154</v>
-      </c>
-      <c r="B2" t="s">
-        <v>155</v>
-      </c>
-      <c r="C2" t="s">
-        <v>156</v>
-      </c>
-      <c r="D2" t="s">
-        <v>157</v>
-      </c>
-      <c r="F2" t="s">
-        <v>49</v>
-      </c>
-      <c r="G2" t="s">
-        <v>37</v>
-      </c>
-      <c r="H2">
+      <c r="G3" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="H3" s="12">
         <v>2026</v>
       </c>
-      <c r="I2" t="s">
-        <v>147</v>
-      </c>
-      <c r="J2" t="s">
-        <v>148</v>
-      </c>
-      <c r="K2" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>159</v>
-      </c>
-      <c r="B3" t="s">
-        <v>160</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="I3" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="J3" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="K3" s="12" t="s">
         <v>161</v>
       </c>
-      <c r="D3" t="s">
-        <v>162</v>
-      </c>
-      <c r="F3" t="s">
-        <v>49</v>
-      </c>
-      <c r="G3" t="s">
-        <v>37</v>
-      </c>
-      <c r="H3">
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="E4" s="11"/>
+      <c r="F4" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="H4" s="11">
         <v>2026</v>
       </c>
-      <c r="I3" t="s">
-        <v>147</v>
-      </c>
-      <c r="J3" t="s">
-        <v>148</v>
-      </c>
-      <c r="K3" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>163</v>
-      </c>
-      <c r="B4" t="s">
-        <v>164</v>
-      </c>
-      <c r="C4" t="s">
-        <v>165</v>
-      </c>
-      <c r="D4" t="s">
-        <v>166</v>
-      </c>
-      <c r="F4" t="s">
-        <v>49</v>
-      </c>
-      <c r="G4" t="s">
-        <v>37</v>
-      </c>
-      <c r="H4">
+      <c r="I4" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="J4" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="K4" s="11" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
+        <v>170</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>172</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>173</v>
+      </c>
+      <c r="E5" s="12"/>
+      <c r="F5" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="H5" s="12">
         <v>2026</v>
       </c>
-      <c r="I4" t="s">
-        <v>147</v>
-      </c>
-      <c r="J4" t="s">
-        <v>148</v>
-      </c>
-      <c r="K4" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>167</v>
-      </c>
-      <c r="B5" t="s">
-        <v>168</v>
-      </c>
-      <c r="C5" t="s">
-        <v>169</v>
-      </c>
-      <c r="D5" t="s">
-        <v>170</v>
-      </c>
-      <c r="F5" t="s">
-        <v>49</v>
-      </c>
-      <c r="G5" t="s">
-        <v>37</v>
-      </c>
-      <c r="H5">
+      <c r="I5" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="J5" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="K5" s="12" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
+        <v>174</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>175</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>176</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>177</v>
+      </c>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="H6" s="11">
         <v>2026</v>
       </c>
-      <c r="I5" t="s">
-        <v>147</v>
-      </c>
-      <c r="J5" t="s">
-        <v>148</v>
-      </c>
-      <c r="K5" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>171</v>
-      </c>
-      <c r="B6" t="s">
-        <v>172</v>
-      </c>
-      <c r="C6" t="s">
-        <v>173</v>
-      </c>
-      <c r="D6" t="s">
-        <v>174</v>
-      </c>
-      <c r="F6" t="s">
-        <v>49</v>
-      </c>
-      <c r="G6" t="s">
-        <v>37</v>
-      </c>
-      <c r="H6">
+      <c r="I6" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="J6" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="K6" s="11" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
+        <v>178</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>180</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>181</v>
+      </c>
+      <c r="E7" s="12"/>
+      <c r="F7" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="H7" s="12">
         <v>2026</v>
       </c>
-      <c r="I6" t="s">
-        <v>147</v>
-      </c>
-      <c r="J6" t="s">
-        <v>148</v>
-      </c>
-      <c r="K6" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>175</v>
-      </c>
-      <c r="B7" t="s">
-        <v>176</v>
-      </c>
-      <c r="C7" t="s">
-        <v>177</v>
-      </c>
-      <c r="D7" t="s">
-        <v>178</v>
-      </c>
-      <c r="F7" t="s">
-        <v>49</v>
-      </c>
-      <c r="G7" t="s">
-        <v>37</v>
-      </c>
-      <c r="H7">
+      <c r="I7" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="J7" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="K7" s="12" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>184</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>185</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>186</v>
+      </c>
+      <c r="E8" s="11"/>
+      <c r="F8" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="G8" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="H8" s="11">
         <v>2026</v>
       </c>
-      <c r="I7" t="s">
-        <v>147</v>
-      </c>
-      <c r="J7" t="s">
-        <v>148</v>
-      </c>
-      <c r="K7" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>180</v>
-      </c>
-      <c r="B8" t="s">
-        <v>181</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="I8" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="J8" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="K8" s="11" t="s">
         <v>182</v>
       </c>
-      <c r="D8" t="s">
-        <v>183</v>
-      </c>
-      <c r="F8" t="s">
-        <v>49</v>
-      </c>
-      <c r="G8" t="s">
-        <v>37</v>
-      </c>
-      <c r="H8">
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" s="12" t="s">
+        <v>187</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>188</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>189</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>190</v>
+      </c>
+      <c r="E9" s="12"/>
+      <c r="F9" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="G9" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="H9" s="12">
         <v>2026</v>
       </c>
-      <c r="I8" t="s">
-        <v>147</v>
-      </c>
-      <c r="J8" t="s">
-        <v>148</v>
-      </c>
-      <c r="K8" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>184</v>
-      </c>
-      <c r="B9" t="s">
-        <v>185</v>
-      </c>
-      <c r="C9" t="s">
-        <v>186</v>
-      </c>
-      <c r="D9" t="s">
-        <v>187</v>
-      </c>
-      <c r="F9" t="s">
-        <v>49</v>
-      </c>
-      <c r="G9" t="s">
-        <v>37</v>
-      </c>
-      <c r="H9">
+      <c r="I9" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="J9" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="K9" s="12" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" s="11" t="s">
+        <v>191</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>192</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>193</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>194</v>
+      </c>
+      <c r="E10" s="11"/>
+      <c r="F10" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="G10" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="H10" s="11">
         <v>2026</v>
       </c>
-      <c r="I9" t="s">
-        <v>147</v>
-      </c>
-      <c r="J9" t="s">
-        <v>148</v>
-      </c>
-      <c r="K9" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>188</v>
-      </c>
-      <c r="B10" t="s">
-        <v>189</v>
-      </c>
-      <c r="C10" t="s">
-        <v>190</v>
-      </c>
-      <c r="D10" t="s">
-        <v>191</v>
-      </c>
-      <c r="F10" t="s">
-        <v>49</v>
-      </c>
-      <c r="G10" t="s">
-        <v>37</v>
-      </c>
-      <c r="H10">
+      <c r="I10" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="J10" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="K10" s="11" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" s="12" t="s">
+        <v>195</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>196</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>197</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>198</v>
+      </c>
+      <c r="E11" s="12"/>
+      <c r="F11" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="G11" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="H11" s="12">
         <v>2026</v>
       </c>
-      <c r="I10" t="s">
-        <v>147</v>
-      </c>
-      <c r="J10" t="s">
-        <v>148</v>
-      </c>
-      <c r="K10" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>192</v>
-      </c>
-      <c r="B11" t="s">
-        <v>193</v>
-      </c>
-      <c r="C11" t="s">
-        <v>194</v>
-      </c>
-      <c r="D11" t="s">
-        <v>195</v>
-      </c>
-      <c r="F11" t="s">
-        <v>49</v>
-      </c>
-      <c r="G11" t="s">
-        <v>37</v>
-      </c>
-      <c r="H11">
-        <v>2026</v>
-      </c>
-      <c r="I11" t="s">
-        <v>147</v>
-      </c>
-      <c r="J11" t="s">
-        <v>148</v>
-      </c>
-      <c r="K11" t="s">
-        <v>179</v>
+      <c r="I11" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="J11" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="K11" s="12" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="12" spans="9:9" x14ac:dyDescent="0.25"/>
@@ -5027,52 +5218,62 @@
       <formula1>"Regular,LEET"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-  <legacyDrawing r:id="rId2"/>
+  <hyperlinks>
+    <hyperlink ref="M1" r:id="rId1" location="#'Start here'!A1"/>
+  </hyperlinks>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D200"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:F200"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="23" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
-        <v>196</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>198</v>
-      </c>
-      <c r="D1" s="3" t="s">
+    <row r="1" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
         <v>199</v>
       </c>
+      <c r="B1" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>200</v>
-      </c>
-      <c r="C2" t="s">
-        <v>201</v>
-      </c>
-      <c r="D2" t="s">
-        <v>37</v>
+      <c r="A2" s="11" t="s">
+        <v>203</v>
+      </c>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11" t="s">
+        <v>204</v>
+      </c>
+      <c r="D2" s="11" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>202</v>
-      </c>
-      <c r="C3" t="s">
-        <v>203</v>
+      <c r="A3" s="12" t="s">
+        <v>205</v>
+      </c>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="4" spans="4:4" x14ac:dyDescent="0.25"/>
@@ -5281,8 +5482,10 @@
       <formula1>'Departments'!$A$2:$A$500</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-  <legacyDrawing r:id="rId2"/>
+  <hyperlinks>
+    <hyperlink ref="F1" r:id="rId1" location="#'Start here'!A1"/>
+  </hyperlinks>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>